<commit_message>
se agrega pedido a la lista de pedidos
</commit_message>
<xml_diff>
--- a/data/datos_negocio.xlsx
+++ b/data/datos_negocio.xlsx
@@ -1012,7 +1012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.8515625" defaultRowHeight="14.4" customHeight="1"/>
   <cols>
     <col width="18.00390625" customWidth="1" min="1" max="1"/>
@@ -1273,6 +1273,65 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="11" t="inlineStr">
+        <is>
+          <t>PED20260618224751</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>2026-06-18 22:47:51</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>+549351000000</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>REP006</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>Filtro de aire</t>
+        </is>
+      </c>
+      <c r="F5" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="G5" s="11" t="n">
+        <v>3200</v>
+      </c>
+      <c r="H5" s="11" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+      <c r="I5" s="11" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="J5" s="11" t="n">
+        <v>3200</v>
+      </c>
+      <c r="K5" s="11" t="n">
+        <v>6400</v>
+      </c>
+      <c r="L5" s="11" t="inlineStr">
+        <is>
+          <t>retiro</t>
+        </is>
+      </c>
+      <c r="M5" s="11" t="inlineStr">
+        <is>
+          <t>CONFIRMADO</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="1" pageOrder="downThenOver"/>

</xml_diff>